<commit_message>
corrección, carga de orígen, asignaturas y marcadores compartidos
</commit_message>
<xml_diff>
--- a/install_root/data_demo/ERASMUS IN.xlsx
+++ b/install_root/data_demo/ERASMUS IN.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Coordenadas" sheetId="1" state="visible" r:id="rId1"/>
@@ -1070,9 +1070,9 @@
           <t>Faculty of Engineering</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>41.0254,28.9470</t>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>41.1052, 29.0250</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alumno 1</t>
+          <t>Alumno HTU 1/2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alumno 2</t>
+          <t>Alumno HTU 1/2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1268,22 +1268,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bases de Datos - I</t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alumno 3</t>
+          <t>Alumno HTU 2/2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unimore</t>
+          <t>HTU</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1315,12 +1315,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Estructura de Computadores - A</t>
+          <t>Bases de Datos - I</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alumno 4</t>
+          <t>Alumno Unimore 1/9</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1362,12 +1362,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fundamentos de Programación II - A</t>
+          <t>Estructura de Computadores - A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alumno 5</t>
+          <t>Alumno Unimore 2/9</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1378,16 +1378,6 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>Unimore</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>un_enlace.pdf</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1409,12 +1399,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Comercio Electrónico</t>
+          <t>Fundamentos de Programación II - A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Alumno 6</t>
+          <t>Alumno Unimore 3/9</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1446,12 +1436,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>Comercio Electrónico</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alumno 7</t>
+          <t>Alumno Unimore 4/9</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1488,17 +1478,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alumno 8</t>
+          <t>Alumno Unimore 5/9</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HTU</t>
+          <t>Unimore</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1520,27 +1515,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>Cálculo y Métodos Numéricos - I</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alumno 9</t>
+          <t>Alumno Unimore 6/9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Alemania</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bonn-Rhein-Sieg</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>x</t>
+          <t>Unimore</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1562,22 +1552,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>(MUII) Sistemas y Servicios en la Nube</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alumno 10</t>
+          <t>Alumno Unimore 7/9</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>UMAG</t>
+          <t>Unimore</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1599,22 +1589,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>Dispositivos y Redes Inalámbricos</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alumno 11</t>
+          <t>Alumno Unimore 8/9</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Duoc UC - Plaza Norte</t>
+          <t>Unimore</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1636,22 +1626,35 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>Gestión de proyectos software</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alumno 12</t>
+          <t>Alumno Unimore 9/9</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Universidad Libre</t>
+          <t>Unimore</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Petra.pdf</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1671,28 +1674,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Calidad de los Sistemas SW</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Alumno 13</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Francia</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>ESAIP</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>2</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1701,7 +1686,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Petra.pdf</t>
+          <t>Petra2.pdf</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1723,22 +1708,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Diseño de Software</t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alumno 14</t>
+          <t>Alumno Bonn-Rhein-Sieg 1/2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ESAIP</t>
+          <t>Bonn-Rhein-Sieg</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1775,37 +1760,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fgbvertb</t>
+          <t>Fundamentos Físicos - I</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alumno 15</t>
+          <t>Alumno Bonn-Rhein-Sieg 2/2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Francia</t>
+          <t>Alemania</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ESAIP</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2</t>
+          <t>Bonn-Rhein-Sieg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>x</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Petra2.pdf</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1825,31 +1800,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Fundamentos Físicos - I</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Alumno 16</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Alemania</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Bonn-Rhein-Sieg</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>Diseño de Software</t>
@@ -1866,25 +1816,40 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="15" customHeight="1" thickBot="1">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cálculo y Métodos Numéricos - I</t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alumno 17</t>
+          <t>Alumno UMAG 1/1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Unimore</t>
+          <t>UMAG</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>C:UsersmariaDownloadsOSSRequestForm-v4.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1906,37 +1871,22 @@
     <row r="19" ht="15" customHeight="1" thickBot="1">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alumno 18</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>C:UsersmariaDownloadsOSSRequestForm-v4.xlsx</t>
+          <t>Alumno Duoc 1/1</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Duoc UC - Plaza Norte</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1958,22 +1908,22 @@
     <row r="20" ht="42" customHeight="1" thickBot="1">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">(MUII) Gestión de Auditoría y Seguridad </t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alumno 19</t>
+          <t>Alumno Universidad Libre 1/1</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Business and Technology University</t>
+          <t>Universidad Libre</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1993,26 +1943,8 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" thickBot="1">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>(MUII) Sistemas y Servicios en la Nube</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Alumno 20</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Unimore</t>
-        </is>
-      </c>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>Estructura de Computadores - A</t>
@@ -2032,22 +1964,22 @@
     <row r="22" ht="15" customHeight="1" thickBot="1">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aceleradores Gráficos</t>
+          <t>Calidad de los Sistemas SW</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alumno 21</t>
+          <t>Alumno ESAIP 1/3</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Udine</t>
+          <t>ESAIP</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2069,22 +2001,22 @@
     <row r="23" ht="15" customHeight="1" thickBot="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Álgebra</t>
+          <t>Diseño de Software</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alumno 22</t>
+          <t>Alumno ESAIP 2/3</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Pol. Milan</t>
+          <t>ESAIP</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2106,22 +2038,22 @@
     <row r="24" ht="28.2" customHeight="1" thickBot="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Álgebra y Matemática Discreta - A</t>
+          <t>fgbvertb</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alumno 23</t>
+          <t>Alumno ESAIP 3/3</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Francia</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Degli Studi di Sassari</t>
+          <t>ESAIP</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2141,26 +2073,8 @@
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" thickBot="1">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Álgebra y Matemática Discreta - I</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Alumno 24</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>University of Petra</t>
-        </is>
-      </c>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Fundamentos de Gestión Empresarial - A</t>
@@ -2180,22 +2094,22 @@
     <row r="26" ht="15" customHeight="1" thickBot="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Arquitectura de Computadores - I</t>
+          <t>Estancia Investigación</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alumno 25</t>
+          <t>Alumno Business 1/4</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Yarmouk University</t>
+          <t>Business and Technology University</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2217,22 +2131,22 @@
     <row r="27" ht="28.2" customHeight="1" thickBot="1">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Auditoría Sistemas Información</t>
+          <t>(MUII) Gestión de Auditoría y Seguridad</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alumno 26</t>
+          <t>Alumno Business 2/4</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Amman Arab University</t>
+          <t>Business and Technology University</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2254,22 +2168,22 @@
     <row r="28" ht="28.2" customHeight="1" thickBot="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bases de Datos - A</t>
+          <t>Diseño Gráfico y Animación</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alumno 27</t>
+          <t>Alumno Business 3/4</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Letonia</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Faculty of Eng. and IT</t>
+          <t>Business and Technology University</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2291,22 +2205,22 @@
     <row r="29" ht="28.2" customHeight="1" thickBot="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bases de Datos - I</t>
+          <t>Organización de Computadores - I</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alumno 28</t>
+          <t>Alumno Business 4/4</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Letonia</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Life Sciences and Tech</t>
+          <t>Business and Technology University</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2326,26 +2240,8 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" thickBot="1">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Cálculo y Métodos Numéricos - I</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Alumno 29</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>TEC</t>
-        </is>
-      </c>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Fundamentos de Programación I - I</t>
@@ -2365,22 +2261,22 @@
     <row r="31" ht="15" customHeight="1" thickBot="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Calidad de los Sistemas SW</t>
+          <t>Aceleradores Gráficos</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alumno 30</t>
+          <t>Alumno Udine 1/2</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Chiapas</t>
+          <t>Udine</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2402,22 +2298,22 @@
     <row r="32" ht="15" customHeight="1" thickBot="1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Comercio Electrónico</t>
+          <t>Estadística - I</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alumno 31</t>
+          <t>Alumno Udine 2/2</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>UA Zacatecas</t>
+          <t>Udine</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2439,22 +2335,22 @@
     <row r="33" ht="15" customHeight="1" thickBot="1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Criptografía</t>
+          <t>Gestión de Sistemas de información</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alumno 32</t>
+          <t>Alumno Udine 2/2</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Nuevo León</t>
+          <t>Udine</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2476,22 +2372,22 @@
     <row r="34" ht="28.2" customHeight="1" thickBot="1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Diseño de Sistemas Interactivos</t>
+          <t>Procesadores de Lenguajes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alumno 33</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
+          <t>Alumno Udine 2/2</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Italia</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Udine</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2511,26 +2407,8 @@
       </c>
     </row>
     <row r="35" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Diseño de Software</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Alumno 34</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
-        </is>
-      </c>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Gestión de proyectos software</t>
@@ -2550,22 +2428,22 @@
     <row r="36" ht="42" customHeight="1" thickBot="1">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Diseño Gráfico y Animación</t>
+          <t>Álgebra</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alumno 35</t>
+          <t>Alumno Pol. Milan 1/3</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Business and Technology University</t>
+          <t>Pol. Milan</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2587,12 +2465,12 @@
     <row r="37" ht="15" customHeight="1" thickBot="1">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Dispositivos y Redes Inalámbricos</t>
+          <t>Estructura de Computadores - A</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alumno 36</t>
+          <t>Alumno Pol. Milan 2/3</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2602,7 +2480,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Unimore</t>
+          <t>Pol. Milan</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2624,12 +2502,12 @@
     <row r="38" ht="15" customHeight="1" thickBot="1">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Estadística - I</t>
+          <t>Ingeniería del Software I - I</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alumno 37</t>
+          <t>Alumno Pol. Milan 3/3</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -2639,7 +2517,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Udine</t>
+          <t>Pol. Milan</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2661,12 +2539,12 @@
     <row r="39" ht="15" customHeight="1" thickBot="1">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Estructura de Computadores - A</t>
+          <t>Procesos de Ingeniería del SW</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alumno 38</t>
+          <t>Alumno Pol. Milan 3/3</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2696,26 +2574,8 @@
       </c>
     </row>
     <row r="40" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Estructura de Computadores - I</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Alumno 39</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Inteligencia Artificial en Videojuegos</t>
@@ -2735,22 +2595,22 @@
     <row r="41" ht="15" customHeight="1" thickBot="1">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Estructura de Datos - A</t>
+          <t>Álgebra y Matemática Discreta - A</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alumno 40</t>
+          <t>Alumno Sassari 1/2</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>University of Petra</t>
+          <t>Degli Studi di Sassari</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2772,22 +2632,30 @@
     <row r="42" ht="15" customHeight="1" thickBot="1">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Estructura de Datos - I</t>
+          <t>Estructura de Computadores - I</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alumno 41</t>
+          <t>Alumno Sassari 2/2</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Yarmouk University</t>
+          <t>Degli Studi di Sassari</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2809,22 +2677,30 @@
     <row r="43" ht="28.2" customHeight="1" thickBot="1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Fundamentos de Gestión Empresarial - A</t>
+          <t>Ingeniería del Software II - I</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alumno 42</t>
+          <t>Alumno Sassari 2/2</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Amman Arab University</t>
+          <t>Degli Studi di Sassari</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2846,22 +2722,30 @@
     <row r="44" ht="28.2" customHeight="1" thickBot="1">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Fundamentos de Gestión Empresarial - B</t>
+          <t>Programación Concurrente y Tiempo Real</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alumno 43</t>
+          <t>Alumno Sassari 2/2</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Letonia</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Faculty of Eng. and IT</t>
+          <t>Degli Studi di Sassari</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2881,26 +2765,8 @@
       </c>
     </row>
     <row r="45" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Fundamentos de Gestión Empresarial - C</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Alumno 44</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Life Sciences and Tech</t>
-        </is>
-      </c>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>Lógica - I</t>
@@ -2920,22 +2786,22 @@
     <row r="46" ht="15" customHeight="1" thickBot="1">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Fundamentos de Gestión Empresarial - I</t>
+          <t>Álgebra y Matemática Discreta - I</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alumno 45</t>
+          <t>Alumno Petra 1/3</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>TEC</t>
+          <t>University of Petra</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2957,22 +2823,22 @@
     <row r="47" ht="15" customHeight="1" thickBot="1">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Fundamentos de Programación I - A</t>
+          <t>Estructura de Datos - A</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alumno 46</t>
+          <t>Alumno Petra 2/3</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Chiapas</t>
+          <t>University of Petra</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2994,22 +2860,22 @@
     <row r="48" ht="15" customHeight="1" thickBot="1">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Fundamentos de Programación I - I</t>
+          <t>Ingeniería Web y de Servicios</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alumno 47</t>
+          <t>Alumno Petra 3/3</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>UA Zacatecas</t>
+          <t>University of Petra</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3031,22 +2897,22 @@
     <row r="49" ht="15" customHeight="1" thickBot="1">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Fundamentos de Programación II - A</t>
+          <t>Programación Declarativa</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alumno 48</t>
+          <t>Alumno Petra 3/3</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Nuevo León</t>
+          <t>University of Petra</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3066,26 +2932,8 @@
       </c>
     </row>
     <row r="50" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Fundamentos de Programación II - I</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Alumno 49</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
-        </is>
-      </c>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="8" t="n"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>Organización de Computadores - I</t>
@@ -3105,22 +2953,22 @@
     <row r="51" ht="28.2" customHeight="1" thickBot="1">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - B</t>
+          <t>Arquitectura de Computadores - I</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alumno 50</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
+          <t>Alumno Yarmouk 1/2</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Jordania</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Yarmouk University</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3142,22 +2990,22 @@
     <row r="52" ht="42" customHeight="1" thickBot="1">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fundamentos Físicos - I</t>
+          <t>Estructura de Datos - I</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alumno 51</t>
+          <t>Alumno Yarmouk 1/2</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Business and Technology University</t>
+          <t>Yarmouk University</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3179,22 +3027,22 @@
     <row r="53" ht="15" customHeight="1" thickBot="1">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Gestión de proyectos software</t>
+          <t>Inteligencia Artificial en Videojuegos</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alumno 52</t>
+          <t>Alumno Yarmouk 2/2</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Unimore</t>
+          <t>Yarmouk University</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3216,22 +3064,22 @@
     <row r="54" ht="15" customHeight="1" thickBot="1">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Gestión de Sistemas de información</t>
+          <t>Redes de Computadores I - A</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alumno 53</t>
+          <t>Alumno Yarmouk 2/2</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Udine</t>
+          <t>Yarmouk University</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3251,26 +3099,8 @@
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" thickBot="1">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Ingeniería del Software I - I</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Alumno 54</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Pol. Milan</t>
-        </is>
-      </c>
+      <c r="C55" s="5" t="n"/>
+      <c r="D55" s="5" t="n"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>Programación Declarativa</t>
@@ -3290,22 +3120,22 @@
     <row r="56" ht="28.2" customHeight="1" thickBot="1">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ingeniería del Software II - I</t>
+          <t>Auditoría Sistemas Información</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alumno 55</t>
+          <t>Alumno Amman 1/2</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Jordania</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Degli Studi di Sassari</t>
+          <t>Amman Arab University</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3327,12 +3157,12 @@
     <row r="57" ht="15" customHeight="1" thickBot="1">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ingeniería Web y de Servicios</t>
+          <t>Fundamentos de Gestión Empresarial - A</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alumno 56</t>
+          <t>Alumno Amman 2/2</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -3342,7 +3172,7 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>University of Petra</t>
+          <t>Amman Arab University</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3364,12 +3194,12 @@
     <row r="58" ht="15" customHeight="1" thickBot="1">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Inteligencia Artificial en Videojuegos</t>
+          <t>Interacción Persona Ordenador I - A</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alumno 57</t>
+          <t>Alumno Amman 2/2</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -3379,7 +3209,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Yarmouk University</t>
+          <t>Amman Arab University</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3401,12 +3231,12 @@
     <row r="59" ht="28.2" customHeight="1" thickBot="1">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Interacción Persona Ordenador I - A</t>
+          <t>Redes de Computadores I - I</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alumno 58</t>
+          <t>Alumno Amman 2/2</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -3436,26 +3266,8 @@
       </c>
     </row>
     <row r="60" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Interacción Persona Ordenador I - B</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Alumno 59</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
+      <c r="C60" s="5" t="n"/>
+      <c r="D60" s="5" t="n"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>Seguridad en redes</t>
@@ -3475,12 +3287,12 @@
     <row r="61" ht="28.2" customHeight="1" thickBot="1">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Interacción Persona Ordenador I - I</t>
+          <t>Bases de Datos - A</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alumno 60</t>
+          <t>Alumno LatviaEng 1/3</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3490,7 +3302,7 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Life Sciences and Tech</t>
+          <t>Faculty of Eng. and IT</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3512,22 +3324,22 @@
     <row r="62" ht="15" customHeight="1" thickBot="1">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Lógica - B</t>
+          <t>Fundamentos de Gestión Empresarial - B</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Alumno 61</t>
+          <t>Alumno LatviaEng 2/3</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Letonia</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>TEC</t>
+          <t>Faculty of Eng. and IT</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3549,22 +3361,22 @@
     <row r="63" ht="15" customHeight="1" thickBot="1">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Lógica - I</t>
+          <t>Interacción Persona Ordenador I - B</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alumno 62</t>
+          <t>Alumno LatviaEng 3/3</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Letonia</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Chiapas</t>
+          <t>Faculty of Eng. and IT</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3584,26 +3396,8 @@
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" thickBot="1">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Metodología de la Programación - A</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Alumno 63</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>UA Zacatecas</t>
-        </is>
-      </c>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>Sistemas Basados en el Conocimiento</t>
@@ -3623,22 +3417,22 @@
     <row r="65" ht="15" customHeight="1" thickBot="1">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Metodología de la Programación - I</t>
+          <t>Bases de Datos - I</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Alumno 64</t>
+          <t>Alumno LatviaLife 1/3</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>Letonia</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Nuevo León</t>
+          <t>Life Sciences and Tech</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3660,22 +3454,22 @@
     <row r="66" ht="28.2" customHeight="1" thickBot="1">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Minería de datos</t>
+          <t>Fundamentos de Gestión Empresarial - C</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Alumno 65</t>
-        </is>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
+          <t>Alumno LatviaLife 2/3</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Letonia</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Life Sciences and Tech</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3697,22 +3491,22 @@
     <row r="67" ht="28.2" customHeight="1" thickBot="1">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Multimedia</t>
+          <t>Interacción Persona Ordenador I - I</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Alumno 66</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D67" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
+          <t>Alumno LatviaLife 3/3</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Letonia</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Life Sciences and Tech</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3732,26 +3526,8 @@
       </c>
     </row>
     <row r="68" ht="42" customHeight="1" thickBot="1">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Organización de Computadores - I</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Alumno 67</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
-        </is>
-      </c>
+      <c r="C68" s="5" t="n"/>
+      <c r="D68" s="5" t="n"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>Sistemas Inteligentes - A</t>
@@ -3771,22 +3547,22 @@
     <row r="69" ht="15" customHeight="1" thickBot="1">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Planificación e Integración de Sistemas</t>
+          <t>Cálculo y Métodos Numéricos - I</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Alumno 68</t>
+          <t>Alumno TEC 1/3</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Unimore</t>
+          <t>TEC</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3808,22 +3584,22 @@
     <row r="70" ht="15" customHeight="1" thickBot="1">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Procesadores de Lenguajes</t>
+          <t>Fundamentos de Gestión Empresarial - I</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Alumno 69</t>
+          <t>Alumno TEC 2/3</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Udine</t>
+          <t>TEC</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3845,22 +3621,22 @@
     <row r="71" ht="15" customHeight="1" thickBot="1">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Procesos de Ingeniería del SW</t>
+          <t>Lógica - B</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Alumno 70</t>
+          <t>Alumno TEC 3/3</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Pol. Milan</t>
+          <t>TEC</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3880,26 +3656,8 @@
       </c>
     </row>
     <row r="72" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Programación Concurrente y Tiempo Real</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Alumno 71</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C72" s="5" t="n"/>
+      <c r="D72" s="5" t="n"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>Sistemas Operativos II</t>
@@ -3919,22 +3677,22 @@
     <row r="73" ht="15" customHeight="1" thickBot="1">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Programación Declarativa</t>
+          <t>Calidad de los Sistemas SW</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Alumno 72</t>
+          <t>Alumno Chiapas 1/2</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>University of Petra</t>
+          <t>Chiapas</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3956,22 +3714,22 @@
     <row r="74" ht="15" customHeight="1" thickBot="1">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Redes de Computadores I - A</t>
+          <t>Fundamentos de Programación I - A</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Alumno 73</t>
+          <t>Alumno Chiapas 1/2</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Yarmouk University</t>
+          <t>Chiapas</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3993,22 +3751,22 @@
     <row r="75" ht="28.2" customHeight="1" thickBot="1">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Redes de Computadores I - I</t>
+          <t>Lógica - I</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Alumno 74</t>
+          <t>Alumno Chiapas 2/2</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Amman Arab University</t>
+          <t>Chiapas</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -4028,26 +3786,8 @@
       </c>
     </row>
     <row r="76" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Robótica Autónoma</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Alumno 75</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
+      <c r="C76" s="5" t="n"/>
+      <c r="D76" s="5" t="n"/>
       <c r="I76" t="inlineStr">
         <is>
           <t>Videojuegos y Realidad Virtual</t>
@@ -4067,22 +3807,22 @@
     <row r="77" ht="28.2" customHeight="1" thickBot="1">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Seguridad de Sistemas Software</t>
+          <t>Comercio Electrónico</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Alumno 76</t>
+          <t>Alumno Zacatecas 1/2</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Letonia</t>
+          <t>México</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Life Sciences and Tech</t>
+          <t>UA Zacatecas</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4104,12 +3844,12 @@
     <row r="78" ht="15" customHeight="1" thickBot="1">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Seguridad en redes</t>
+          <t>Fundamentos de Programación I - I</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Alumno 77</t>
+          <t>Alumno Zacatecas 1/2</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -4119,19 +3859,19 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>TEC</t>
+          <t>UA Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" thickBot="1">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Seguridad en Sistemas Informáticos</t>
+          <t>Metodología de la Programación - A</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Alumno 78</t>
+          <t>Alumno Zacatecas 2/2</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
@@ -4141,41 +3881,23 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Chiapas</t>
+          <t>UA Zacatecas</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" thickBot="1">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Sistemas  Distribuidos -  B</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Alumno 79</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>UA Zacatecas</t>
-        </is>
-      </c>
+      <c r="C80" s="5" t="n"/>
+      <c r="D80" s="5" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" thickBot="1">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Sistemas  Distribuidos - A</t>
+          <t>Criptografía</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Alumno 80</t>
+          <t>Alumno Leon 1/2</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -4192,1332 +3914,393 @@
     <row r="82" ht="28.2" customHeight="1" thickBot="1">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Fundamentos de Programación II - A</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Alumno 81</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
+          <t>Alumno Leon 1/2</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
         </is>
       </c>
     </row>
     <row r="83" ht="28.2" customHeight="1" thickBot="1">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Metodología de la Programación - I</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Alumno 82</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D83" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
+          <t>Alumno Leon 2/2</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>México</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Nuevo León</t>
         </is>
       </c>
     </row>
     <row r="84" ht="42" customHeight="1" thickBot="1">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Alumno 83</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
+      <c r="C84" s="5" t="n"/>
+      <c r="D84" s="5" t="n"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" thickBot="1">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Diseño de Sistemas Interactivos</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Alumno 84</t>
+          <t>Alumno TurkeyEng 1/2</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Unimore</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>x</t>
+          <t>Faculty of Engineering</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" thickBot="1">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Fundamentos de Programación II - I</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Alumno 85</t>
+          <t>Alumno TurkeyEng 1/2</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Udine</t>
+          <t>Faculty of Engineering</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" thickBot="1">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Minería de datos</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Alumno 86</t>
+          <t>Alumno TurkeyEng 2/2</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Pol. Milan</t>
+          <t>Faculty of Engineering</t>
         </is>
       </c>
     </row>
     <row r="88" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Alumno 87</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C88" s="5" t="n"/>
+      <c r="D88" s="5" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" thickBot="1">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Diseño de Software</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Alumno 88</t>
+          <t>Alumno Kadir 1/3</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>University of Petra</t>
+          <t>Kadir Has University</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" thickBot="1">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Fundamentos Físicos - B</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Alumno 89</t>
+          <t>Alumno Kadir 2/3</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Yarmouk University</t>
+          <t>Kadir Has University</t>
         </is>
       </c>
     </row>
     <row r="91" ht="28.2" customHeight="1" thickBot="1">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Estancia Investigación</t>
+          <t>Multimedia</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Alumno 90</t>
+          <t>Alumno Kadir 3/3</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Jordania</t>
+          <t>Turquía</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Amman Arab University</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Alumno 91</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
-    </row>
+          <t>Kadir Has University</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="28.2" customHeight="1" thickBot="1"/>
     <row r="93" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Alumno 92</t>
-        </is>
-      </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>Life Sciences and Tech</t>
-        </is>
-      </c>
+      <c r="C93" s="5" t="n"/>
+      <c r="D93" s="5" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" thickBot="1">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Alumno 93</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>TEC</t>
-        </is>
-      </c>
+      <c r="C94" s="5" t="n"/>
+      <c r="D94" s="5" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" thickBot="1">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Alumno 94</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>Chiapas</t>
-        </is>
-      </c>
+      <c r="C95" s="5" t="n"/>
+      <c r="D95" s="5" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" thickBot="1">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Alumno 95</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>UA Zacatecas</t>
-        </is>
-      </c>
+      <c r="C96" s="5" t="n"/>
+      <c r="D96" s="5" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" thickBot="1">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Alumno 96</t>
-        </is>
-      </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
+      <c r="C97" s="5" t="n"/>
+      <c r="D97" s="5" t="n"/>
     </row>
     <row r="98" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Alumno 97</t>
-        </is>
-      </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
-        </is>
-      </c>
+      <c r="C98" s="5" t="n"/>
+      <c r="D98" s="5" t="n"/>
     </row>
     <row r="99" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Alumno 98</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D99" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
-        </is>
-      </c>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="8" t="n"/>
     </row>
     <row r="100" ht="42" customHeight="1" thickBot="1">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Alumno 99</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
-        </is>
-      </c>
+      <c r="C100" s="5" t="n"/>
+      <c r="D100" s="5" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" thickBot="1">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Alumno 100</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>Unimore</t>
-        </is>
-      </c>
+      <c r="C101" s="5" t="n"/>
+      <c r="D101" s="5" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" thickBot="1">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Alumno 101</t>
-        </is>
-      </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="inlineStr">
-        <is>
-          <t>Udine</t>
-        </is>
-      </c>
+      <c r="C102" s="5" t="n"/>
+      <c r="D102" s="5" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" thickBot="1">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Alumno 102</t>
-        </is>
-      </c>
-      <c r="C103" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D103" s="5" t="inlineStr">
-        <is>
-          <t>Pol. Milan</t>
-        </is>
-      </c>
+      <c r="C103" s="5" t="n"/>
+      <c r="D103" s="5" t="n"/>
     </row>
     <row r="104" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Alumno 103</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C104" s="5" t="n"/>
+      <c r="D104" s="5" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" thickBot="1">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Alumno 104</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D105" s="5" t="inlineStr">
-        <is>
-          <t>University of Petra</t>
-        </is>
-      </c>
+      <c r="C105" s="5" t="n"/>
+      <c r="D105" s="5" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" thickBot="1">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Alumno 105</t>
-        </is>
-      </c>
-      <c r="C106" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D106" s="5" t="inlineStr">
-        <is>
-          <t>Yarmouk University</t>
-        </is>
-      </c>
+      <c r="C106" s="5" t="n"/>
+      <c r="D106" s="5" t="n"/>
     </row>
     <row r="107" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Alumno 106</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
-        <is>
-          <t>Amman Arab University</t>
-        </is>
-      </c>
+      <c r="C107" s="5" t="n"/>
+      <c r="D107" s="5" t="n"/>
     </row>
     <row r="108" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Alumno 107</t>
-        </is>
-      </c>
-      <c r="C108" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D108" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
+      <c r="C108" s="5" t="n"/>
+      <c r="D108" s="5" t="n"/>
     </row>
     <row r="109" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Alumno 108</t>
-        </is>
-      </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D109" s="5" t="inlineStr">
-        <is>
-          <t>Life Sciences and Tech</t>
-        </is>
-      </c>
+      <c r="C109" s="5" t="n"/>
+      <c r="D109" s="5" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1" thickBot="1">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Alumno 109</t>
-        </is>
-      </c>
-      <c r="C110" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D110" s="5" t="inlineStr">
-        <is>
-          <t>TEC</t>
-        </is>
-      </c>
+      <c r="C110" s="5" t="n"/>
+      <c r="D110" s="5" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1" thickBot="1">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Alumno 110</t>
-        </is>
-      </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D111" s="5" t="inlineStr">
-        <is>
-          <t>Chiapas</t>
-        </is>
-      </c>
+      <c r="C111" s="5" t="n"/>
+      <c r="D111" s="5" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1" thickBot="1">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Alumno 111</t>
-        </is>
-      </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D112" s="5" t="inlineStr">
-        <is>
-          <t>UA Zacatecas</t>
-        </is>
-      </c>
+      <c r="C112" s="5" t="n"/>
+      <c r="D112" s="5" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1" thickBot="1">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Alumno 112</t>
-        </is>
-      </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D113" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
+      <c r="C113" s="5" t="n"/>
+      <c r="D113" s="5" t="n"/>
     </row>
     <row r="114" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Alumno 113</t>
-        </is>
-      </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D114" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
-        </is>
-      </c>
+      <c r="C114" s="5" t="n"/>
+      <c r="D114" s="5" t="n"/>
     </row>
     <row r="115" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Estancia Investigación</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Alumno 114</t>
-        </is>
-      </c>
-      <c r="C115" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D115" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
-        </is>
-      </c>
+      <c r="C115" s="6" t="n"/>
+      <c r="D115" s="8" t="n"/>
     </row>
     <row r="116" ht="42" customHeight="1" thickBot="1">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Seguridad de Sistemas Software</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Alumno 115</t>
-        </is>
-      </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
-        </is>
-      </c>
+      <c r="C116" s="5" t="n"/>
+      <c r="D116" s="5" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1" thickBot="1">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Seguridad en redes</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Alumno 116</t>
-        </is>
-      </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D117" s="5" t="inlineStr">
-        <is>
-          <t>Unimore</t>
-        </is>
-      </c>
+      <c r="C117" s="5" t="n"/>
+      <c r="D117" s="5" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1" thickBot="1">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Seguridad en Sistemas Informáticos</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Alumno 117</t>
-        </is>
-      </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D118" s="5" t="inlineStr">
-        <is>
-          <t>Udine</t>
-        </is>
-      </c>
+      <c r="C118" s="5" t="n"/>
+      <c r="D118" s="5" t="n"/>
     </row>
     <row r="119" ht="15" customHeight="1" thickBot="1">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Sistemas  Distribuidos -  B</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Alumno 118</t>
-        </is>
-      </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D119" s="5" t="inlineStr">
-        <is>
-          <t>Pol. Milan</t>
-        </is>
-      </c>
+      <c r="C119" s="5" t="n"/>
+      <c r="D119" s="5" t="n"/>
     </row>
     <row r="120" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Sistemas  Distribuidos - A</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Alumno 119</t>
-        </is>
-      </c>
-      <c r="C120" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D120" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C120" s="5" t="n"/>
+      <c r="D120" s="5" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" thickBot="1">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Sistemas Basados en el Conocimiento</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Alumno 120</t>
-        </is>
-      </c>
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D121" s="5" t="inlineStr">
-        <is>
-          <t>University of Petra</t>
-        </is>
-      </c>
+      <c r="C121" s="5" t="n"/>
+      <c r="D121" s="5" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" thickBot="1">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Sistemas de Información - A</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Alumno 121</t>
-        </is>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="inlineStr">
-        <is>
-          <t>Yarmouk University</t>
-        </is>
-      </c>
+      <c r="C122" s="5" t="n"/>
+      <c r="D122" s="5" t="n"/>
     </row>
     <row r="123" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Sistemas de Información - I</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Alumno 122</t>
-        </is>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="inlineStr">
-        <is>
-          <t>Amman Arab University</t>
-        </is>
-      </c>
+      <c r="C123" s="5" t="n"/>
+      <c r="D123" s="5" t="n"/>
     </row>
     <row r="124" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>Sistemas Empotrados</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Alumno 123</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
+      <c r="C124" s="5" t="n"/>
+      <c r="D124" s="5" t="n"/>
     </row>
     <row r="125" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Sistemas Inteligentes - A</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Alumno 124</t>
-        </is>
-      </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>Life Sciences and Tech</t>
-        </is>
-      </c>
+      <c r="C125" s="5" t="n"/>
+      <c r="D125" s="5" t="n"/>
     </row>
     <row r="126" ht="15" customHeight="1" thickBot="1">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Sistemas Inteligentes - I</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Alumno 125</t>
-        </is>
-      </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>TEC</t>
-        </is>
-      </c>
+      <c r="C126" s="5" t="n"/>
+      <c r="D126" s="5" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1" thickBot="1">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Sistemas Multiagentes</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Alumno 126</t>
-        </is>
-      </c>
-      <c r="C127" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D127" s="5" t="inlineStr">
-        <is>
-          <t>Chiapas</t>
-        </is>
-      </c>
+      <c r="C127" s="5" t="n"/>
+      <c r="D127" s="5" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1" thickBot="1">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Sistemas Operativos I - A</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Alumno 127</t>
-        </is>
-      </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D128" s="5" t="inlineStr">
-        <is>
-          <t>UA Zacatecas</t>
-        </is>
-      </c>
+      <c r="C128" s="5" t="n"/>
+      <c r="D128" s="5" t="n"/>
     </row>
     <row r="129" ht="15" customHeight="1" thickBot="1">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Sistemas Operativos II</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Alumno 128</t>
-        </is>
-      </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>México</t>
-        </is>
-      </c>
-      <c r="D129" s="5" t="inlineStr">
-        <is>
-          <t>Nuevo León</t>
-        </is>
-      </c>
+      <c r="C129" s="5" t="n"/>
+      <c r="D129" s="5" t="n"/>
     </row>
     <row r="130" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Tecnología de Computadores - B</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Alumno 129</t>
-        </is>
-      </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D130" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Engineering</t>
-        </is>
-      </c>
+      <c r="C130" s="5" t="n"/>
+      <c r="D130" s="5" t="n"/>
     </row>
     <row r="131" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Tecnologías y sistemas web</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Alumno 130</t>
-        </is>
-      </c>
-      <c r="C131" s="6" t="inlineStr">
-        <is>
-          <t>Turquía</t>
-        </is>
-      </c>
-      <c r="D131" s="8" t="inlineStr">
-        <is>
-          <t>Kadir Has University</t>
-        </is>
-      </c>
+      <c r="C131" s="6" t="n"/>
+      <c r="D131" s="8" t="n"/>
     </row>
     <row r="132" ht="42" customHeight="1" thickBot="1">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>Teoría de Autómatas y Computación</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>Alumno 131</t>
-        </is>
-      </c>
-      <c r="C132" s="5" t="inlineStr">
-        <is>
-          <t>Georgia</t>
-        </is>
-      </c>
-      <c r="D132" s="5" t="inlineStr">
-        <is>
-          <t>Business and Technology University</t>
-        </is>
-      </c>
+      <c r="C132" s="5" t="n"/>
+      <c r="D132" s="5" t="n"/>
     </row>
     <row r="133" ht="15" customHeight="1" thickBot="1">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>Videojuegos y Realidad Virtual</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Alumno 132</t>
-        </is>
-      </c>
-      <c r="C133" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D133" s="5" t="inlineStr">
-        <is>
-          <t>Unimore</t>
-        </is>
-      </c>
+      <c r="C133" s="5" t="n"/>
+      <c r="D133" s="5" t="n"/>
     </row>
     <row r="134" ht="15" customHeight="1" thickBot="1">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Visión artificial y reconocimiento de patrones</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>Alumno 133</t>
-        </is>
-      </c>
-      <c r="C134" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D134" s="5" t="inlineStr">
-        <is>
-          <t>Udine</t>
-        </is>
-      </c>
+      <c r="C134" s="5" t="n"/>
+      <c r="D134" s="5" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1" thickBot="1">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>Seguridad de Sistemas Software</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>Alumno 134</t>
-        </is>
-      </c>
-      <c r="C135" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D135" s="5" t="inlineStr">
-        <is>
-          <t>Pol. Milan</t>
-        </is>
-      </c>
+      <c r="C135" s="5" t="n"/>
+      <c r="D135" s="5" t="n"/>
     </row>
     <row r="136" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Seguridad en redes</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Alumno 135</t>
-        </is>
-      </c>
-      <c r="C136" s="5" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D136" s="5" t="inlineStr">
-        <is>
-          <t>Degli Studi di Sassari</t>
-        </is>
-      </c>
+      <c r="C136" s="5" t="n"/>
+      <c r="D136" s="5" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1" thickBot="1">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Seguridad en Sistemas Informáticos</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Alumno 136</t>
-        </is>
-      </c>
-      <c r="C137" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D137" s="5" t="inlineStr">
-        <is>
-          <t>University of Petra</t>
-        </is>
-      </c>
+      <c r="C137" s="5" t="n"/>
+      <c r="D137" s="5" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" thickBot="1">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>Sistemas  Distribuidos -  B</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>Alumno 137</t>
-        </is>
-      </c>
-      <c r="C138" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D138" s="5" t="inlineStr">
-        <is>
-          <t>Yarmouk University</t>
-        </is>
-      </c>
+      <c r="C138" s="5" t="n"/>
+      <c r="D138" s="5" t="n"/>
     </row>
     <row r="139" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>Sistemas  Distribuidos - A</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>Alumno 138</t>
-        </is>
-      </c>
-      <c r="C139" s="5" t="inlineStr">
-        <is>
-          <t>Jordania</t>
-        </is>
-      </c>
-      <c r="D139" s="5" t="inlineStr">
-        <is>
-          <t>Amman Arab University</t>
-        </is>
-      </c>
+      <c r="C139" s="5" t="n"/>
+      <c r="D139" s="5" t="n"/>
     </row>
     <row r="140" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Sistemas Basados en el Conocimiento</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>Alumno 139</t>
-        </is>
-      </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D140" s="5" t="inlineStr">
-        <is>
-          <t>Faculty of Eng. and IT</t>
-        </is>
-      </c>
+      <c r="C140" s="5" t="n"/>
+      <c r="D140" s="5" t="n"/>
     </row>
     <row r="141" ht="28.2" customHeight="1" thickBot="1">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Sistemas de Información - A</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Alumno 140</t>
-        </is>
-      </c>
-      <c r="C141" s="5" t="inlineStr">
-        <is>
-          <t>Letonia</t>
-        </is>
-      </c>
-      <c r="D141" s="5" t="inlineStr">
-        <is>
-          <t>Life Sciences and Tech</t>
-        </is>
-      </c>
+      <c r="C141" s="5" t="n"/>
+      <c r="D141" s="5" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J77">

</xml_diff>